<commit_message>
Completa la plantilla de Biomédica y el indicador del plan en BACPPlanner
La plantilla de Ingeniería Civil Biomédica 2019 traía "[COMPLETAR nº de
niveles]" y una hoja Parametros que la app no leía; ahora declara los 11
semestres que dan las mallas oficiales de la USACH, citadas en el
README, y la app la carga como plan válido. Los 40 ramos de especialidad
van solo con su código, porque la malla oficial no dice qué nombre
corresponde a cada código. El indicador superior ya no vuelve a "Sin
plan cargado" después de cargar un plan.

Verificación en Chromium: la plantilla carga con 55 asignaturas y 11
semestres, los ramos sin nombre muestran su código y el indicador
mantiene el plan al cambiar de idioma.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014pCufsSyMrFHacLzmDwGqp
</commit_message>
<xml_diff>
--- a/BACPPlanner/mallas_ejemplo/Civil/PLANTILLA_Ing_Civil_Biomedica_2019.xlsx
+++ b/BACPPlanner/mallas_ejemplo/Civil/PLANTILLA_Ing_Civil_Biomedica_2019.xlsx
@@ -537,11 +537,7 @@
           <t>94000</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
@@ -654,11 +650,7 @@
           <t>94001</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
@@ -721,11 +713,7 @@
           <t>94002</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -738,11 +726,7 @@
           <t>94003</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
@@ -780,11 +764,7 @@
           <t>94004</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
@@ -822,11 +802,7 @@
           <t>94005</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
@@ -839,11 +815,7 @@
           <t>94006</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
@@ -856,11 +828,7 @@
           <t>94007</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
@@ -873,11 +841,7 @@
           <t>94008</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
@@ -940,11 +904,7 @@
           <t>94009</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -957,11 +917,7 @@
           <t>94010</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
@@ -974,11 +930,7 @@
           <t>94011</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
@@ -991,11 +943,7 @@
           <t>94012</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
@@ -1008,11 +956,7 @@
           <t>94013</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
@@ -1050,11 +994,7 @@
           <t>94014</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
@@ -1067,11 +1007,7 @@
           <t>94015</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
@@ -1084,11 +1020,7 @@
           <t>94016</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
@@ -1101,11 +1033,7 @@
           <t>94017</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
@@ -1118,11 +1046,7 @@
           <t>94018</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
@@ -1160,11 +1084,7 @@
           <t>94019</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
@@ -1177,11 +1097,7 @@
           <t>94020</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
@@ -1194,11 +1110,7 @@
           <t>94021</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
@@ -1211,11 +1123,7 @@
           <t>94022</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
@@ -1228,11 +1136,7 @@
           <t>94023</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
@@ -1245,11 +1149,7 @@
           <t>94024</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
@@ -1262,11 +1162,7 @@
           <t>94025</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
@@ -1279,11 +1175,7 @@
           <t>94026</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
@@ -1296,11 +1188,7 @@
           <t>94027</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
@@ -1313,11 +1201,7 @@
           <t>94028</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
@@ -1330,11 +1214,7 @@
           <t>94029</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
@@ -1347,11 +1227,7 @@
           <t>94030</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
@@ -1364,11 +1240,7 @@
           <t>94031</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
@@ -1381,11 +1253,7 @@
           <t>94032</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
@@ -1398,11 +1266,7 @@
           <t>94033</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
@@ -1415,11 +1279,7 @@
           <t>94034</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
@@ -1432,11 +1292,7 @@
           <t>94035</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
@@ -1449,11 +1305,7 @@
           <t>94036</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
@@ -1466,11 +1318,7 @@
           <t>94037</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
@@ -1483,11 +1331,7 @@
           <t>94038</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
@@ -1500,11 +1344,7 @@
           <t>94039</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>[COMPLETAR — ramo de especialidad]</t>
-        </is>
-      </c>
+      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
@@ -1548,31 +1388,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>parametro</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>periodos</t>
+          <t>valor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Ingeniería Civil Biomédica 2019</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>[COMPLETAR nº de niveles]</t>
-        </is>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>periodos</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1592,7 +1442,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>PLANTILLA — Ingeniería Civil Biomédica 2019 (PDF escaneado, no legible por OCR).</t>
+          <t>PLANTILLA: Ingeniería Civil Biomédica 2019 (PDF escaneado, no legible por OCR).</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1484,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rellena 'periodo' (nivel) en cada fila y 'periodos' en la hoja Parametros.</t>
+          <t>Rellena 'periodo' (nivel) en cada fila.</t>
         </is>
       </c>
     </row>

</xml_diff>